<commit_message>
feat(diaries): production-ready daily, district, and phq diaries with accused history (PI/PO/BC)
</commit_message>
<xml_diff>
--- a/python_worker/templates/Daily_Diary_16Jul2026_AllStations.xlsx
+++ b/python_worker/templates/Daily_Diary_16Jul2026_AllStations.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -571,53 +571,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PS Parliament Street</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>FIR/2026/1007</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>NDPS Act Sec 379</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Amit Jain S/O Mohan Jain R/O 107, Janpath, New Delhi - 110001</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>16/07/2026 21:49</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Street 7, Janpath, New Delhi</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Complaint received from complainant. Janpath area. Police reached scene and registered FIR. Investigation ongoing.</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Manj @Mannu S/O Shakuntla Devi R/O 236, Jahangirpuri, New Delhi</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>SI Gupta (PIS PIS10007)</t>
-        </is>
-      </c>
-    </row>
+    <row r="5" ht="18" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A4:I5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -630,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -699,46 +653,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Mohan Lal S/O Hari Lal R/O 65, Connaught Place, Delhi Age- 40 yrs</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>FIR/2026/1015</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>IPC Sec 302</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>PS Parliament Street</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Inspector Insp. Sharma</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>9820000165</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>judicial_custody</t>
-        </is>
-      </c>
-    </row>
+    <row r="5" ht="18" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A4:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -751,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -805,13 +720,6 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Disposal (Challan / Untrace / Cancel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
         </is>
       </c>
     </row>
@@ -829,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -883,13 +791,6 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Disposal (Challan / Untrace / Cancel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
         </is>
       </c>
     </row>
@@ -907,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -961,13 +862,6 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Disposal (Challan / Untrace / Cancel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
         </is>
       </c>
     </row>
@@ -985,7 +879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1065,56 +959,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>DD/2026/5024</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>25/05/2026</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Mohan Yadav</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>34, Sector-4, Rohini, Delhi</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>25/05/2026</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>SI Tiwari</t>
-        </is>
-      </c>
-    </row>
+    <row r="5" ht="18" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A4:J5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1127,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1202,51 +1047,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>DD/2026/6026</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>16/07/2026</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Near isolated plot Sadar Bazar, Delhi</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>27/05/2026</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>47-57 yrs</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Insp. Verma</t>
-        </is>
-      </c>
-    </row>
+    <row r="5" ht="18" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A4:I5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1259,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1328,13 +1129,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
@@ -1349,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1402,13 +1196,6 @@
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Name of IO (Rank / Name / PIS No.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1501,13 +1288,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1519,7 +1299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1588,13 +1368,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -1609,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1696,13 +1469,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1714,7 +1480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1777,31 +1543,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>PS Parliament Street</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="5" ht="18" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A4:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1814,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1900,13 +1642,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1918,7 +1653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2005,13 +1740,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2023,7 +1751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2121,13 +1849,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2139,7 +1860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2218,13 +1939,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2236,7 +1950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2310,13 +2024,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2328,7 +2035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="3"/>
@@ -2406,311 +2113,28 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="4" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="4" t="n"/>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="6" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="6" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="4" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="6" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="4" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="6" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
-      <c r="J20" s="4" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" s="4" t="n"/>
-      <c r="I21" s="4" t="n"/>
-      <c r="J21" s="6" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="n"/>
-      <c r="J22" s="4" t="n"/>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
-      <c r="I23" s="4" t="n"/>
-      <c r="J23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="4" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
-      <c r="I25" s="4" t="n"/>
-      <c r="J25" s="6" t="n"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
-    </row>
+    <row r="5" ht="18" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="18" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1"/>
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1"/>
+    <row r="24" ht="18" customHeight="1"/>
+    <row r="25" ht="18" customHeight="1"/>
+    <row r="26" ht="18" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2722,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2789,13 +2213,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>No records for this date.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>